<commit_message>
Update Member_B_length sheet to match length_cases.csv
</commit_message>
<xml_diff>
--- a/docs/Task3_Test_Cases.xlsx
+++ b/docs/Task3_Test_Cases.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Azka Nadeem\validators\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D8025CE-B70B-4F42-A709-68DDED49BA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="9000"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Member_A_ipv4" sheetId="1" r:id="rId1"/>
@@ -19,8 +25,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -28,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="74">
   <si>
     <t>Test ID</t>
   </si>
@@ -232,19 +236,31 @@
   </si>
   <si>
     <t>assignment_tests/member_b/test_b_csv_length.py::test_length_from_csv[TC_B07]</t>
+  </si>
+  <si>
+    <t>TC_B08</t>
+  </si>
+  <si>
+    <t>TC_B09</t>
+  </si>
+  <si>
+    <t>text="", min=0, max=0</t>
+  </si>
+  <si>
+    <t>assignment_tests/member_b/test_b_csv_length.py::test_length_from_csv[TC_B08]</t>
+  </si>
+  <si>
+    <t>text="a", min=0, max=0</t>
+  </si>
+  <si>
+    <t>assignment_tests/member_b/test_b_csv_length.py::test_length_from_csv[TC_B09]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="23">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -265,158 +281,13 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="8"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -429,194 +300,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -624,251 +309,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -879,61 +322,17 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1218,14 +617,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -1270,7 +669,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="27.6" spans="1:10">
+    <row r="2" spans="1:10" ht="28">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1302,7 +701,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" ht="27.6" spans="1:10">
+    <row r="3" spans="1:10" ht="28">
       <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
@@ -1334,7 +733,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" ht="27.6" spans="1:10">
+    <row r="4" spans="1:10" ht="28">
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
@@ -1366,7 +765,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" ht="27.6" spans="1:10">
+    <row r="5" spans="1:10" ht="28">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
@@ -1398,7 +797,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" ht="27.6" spans="1:10">
+    <row r="6" spans="1:10" ht="28">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -1430,7 +829,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" ht="27.6" spans="1:10">
+    <row r="7" spans="1:10" ht="28">
       <c r="A7" s="2" t="s">
         <v>34</v>
       </c>
@@ -1462,7 +861,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" ht="27.6" spans="1:10">
+    <row r="8" spans="1:10" ht="28">
       <c r="A8" s="2" t="s">
         <v>37</v>
       </c>
@@ -1494,7 +893,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" ht="27.6" spans="1:10">
+    <row r="9" spans="1:10" ht="28">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -1528,15 +927,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -1581,7 +978,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="27.6" spans="1:10">
+    <row r="2" spans="1:10" ht="28">
       <c r="A2" s="2" t="s">
         <v>43</v>
       </c>
@@ -1613,7 +1010,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" ht="27.6" spans="1:10">
+    <row r="3" spans="1:10" ht="28">
       <c r="A3" s="2" t="s">
         <v>50</v>
       </c>
@@ -1645,7 +1042,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" ht="27.6" spans="1:10">
+    <row r="4" spans="1:10" ht="28">
       <c r="A4" s="2" t="s">
         <v>53</v>
       </c>
@@ -1677,7 +1074,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" ht="27.6" spans="1:10">
+    <row r="5" spans="1:10" ht="28">
       <c r="A5" s="2" t="s">
         <v>56</v>
       </c>
@@ -1709,7 +1106,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" ht="27.6" spans="1:10">
+    <row r="6" spans="1:10" ht="28">
       <c r="A6" s="2" t="s">
         <v>59</v>
       </c>
@@ -1741,7 +1138,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" ht="27.6" spans="1:10">
+    <row r="7" spans="1:10" ht="28">
       <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
@@ -1773,7 +1170,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" ht="27.6" spans="1:10">
+    <row r="8" spans="1:10" ht="28">
       <c r="A8" s="2" t="s">
         <v>65</v>
       </c>
@@ -1805,8 +1202,72 @@
         <v>19</v>
       </c>
     </row>
+    <row r="9" spans="1:10" ht="28">
+      <c r="A9" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="28">
+      <c r="A10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" t="s">
+        <v>72</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>